<commit_message>
feat: adiciona modulo collector para ingestao de comentarios reais
</commit_message>
<xml_diff>
--- a/analise_forum/resultados/resultados_analise.xlsx
+++ b/analise_forum/resultados/resultados_analise.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,21 +450,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>O portal &lt;a href='link'&gt;portal.univ.edu&lt;/a&gt; tá travado de novo!! @suporte resolve isso por favor 😡</t>
+          <t>O filme é simplesmente espetacular! Atuações impecáveis e direção fantástica. Recomendo muito! 🎬✨</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>O portal portalunivedu tá travado de novo resolve isso por favor</t>
+          <t>O filme é simplesmente espetacular Atuações impecáveis e direção fantástica Recomendo muito</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.9817</v>
+        <v>0.9883</v>
       </c>
     </row>
     <row r="3">
@@ -473,21 +473,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>**Excelente** a aula de hoje! Os slides ajudaram bastante. Valeu @caio_monitor 🙌✨</t>
+          <t>Péssima experiência no fórum hoje, ninguém responde minhas dúvidas e o suporte é terrível... 😡</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Excelente a aula de hoje Os slides ajudaram bastante Valeu</t>
+          <t>Péssima experiência no fórum hoje ninguém responde minhas dúvidas e o suporte é terrível</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>admiration</t>
+          <t>disgust</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.9455</v>
+        <v>0.5688</v>
       </c>
     </row>
     <row r="4">
@@ -496,21 +496,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>estou   totalmente   perdido   no   trabalho...   alguém   pode   me   ajudar??? #ajuda</t>
+          <t>Achei a aula muito didática, os exemplos práticos ajudaram demais a entender o conteúdo. Valeu monitor!</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>estou totalmente perdido no trabalho alguém pode me ajudar</t>
+          <t>Achei a aula muito didática os exemplos práticos ajudaram demais a entender o conteúdo Valeu monitor</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>sadness</t>
+          <t>gratitude</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.9025</v>
+        <v>0.9766</v>
       </c>
     </row>
     <row r="5">
@@ -519,21 +519,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gente, adiaram a data de entrega para a próxima sexta!! 🎉🎉🎉 www.forum.edu/avisos @todos</t>
+          <t>Estou completamente frustrado com esse trabalho. O enunciado tá confuso e nada funciona como deveria. #desespero</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gente adiaram a data de entrega para a próxima sexta</t>
+          <t>Estou completamente frustrado com esse trabalho O enunciado tá confuso e nada funciona como deveria</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>anger</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.986</v>
+        <v>0.6840000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -542,21 +542,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>@maria_123 acho que vou reprovar nessa matéria... tô bem desanimado 😔</t>
+          <t>Gente, adiando a entrega do projeto para semana que vem! Sensacional demais, deu um alívio enorme 🎉</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>acho que vou reprovar nessa matéria tô bem desanimado</t>
+          <t>Gente adiando a entrega do projeto para semana que vem Sensacional demais deu um alívio enorme</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>sadness</t>
+          <t>realization</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.8951</v>
+        <v>0.1977</v>
       </c>
     </row>
     <row r="7">
@@ -565,21 +565,573 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alguém sabe se o laboratório de IA vai estar aberto amanhã? `python main.py`</t>
+          <t>O aplicativo vive travando na hora de fazer o login. Decepcionado com a última atualização.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Alguém sabe se o laboratório de IA vai estar aberto amanhã python mainpy</t>
+          <t>O aplicativo vive travando na hora de fazer o login Decepcionado com a última atualização</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>curiosity</t>
+          <t>disappointment</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.5968</v>
+        <v>0.9316</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Alguém mais com dificuldade na matéria de IA? Tô achando o conteúdo bem puxado este semestre... 😔</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Alguém mais com dificuldade na matéria de IA Tô achando o conteúdo bem puxado este semestre</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9375</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Incrível como a comunidade se ajuda aqui! Consegui resolver o bug no código em 5 minutos. Muito obrigado a todos!</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Incrível como a comunidade se ajuda aqui Consegui resolver o bug no código em minutos Muito obrigado a todos</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>gratitude</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.9896</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Horrível, não percam o tempo de vocês assistindo esse filme. O final não faz sentido nenhum.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Horrível não percam o tempo de vocês assistindo esse filme O final não faz sentido nenhum</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>disgust</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.8726</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tô super animado com o novo projeto da disciplina! Tem tudo pra ser uma experiência sensacional. 🚀</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Tô super animado com o novo projeto da disciplina Tem tudo pra ser uma experiência sensacional</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>excitement</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9445</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>O filme é simplesmente espetacular! Atuações impecáveis e direção fantástica. Recomendo muito! 🎬✨</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>O filme é simplesmente espetacular Atuações impecáveis e direção fantástica Recomendo muito</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.9883</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Péssima experiência no fórum hoje, ninguém responde minhas dúvidas e o suporte é terrível... 😡</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Péssima experiência no fórum hoje ninguém responde minhas dúvidas e o suporte é terrível</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>disgust</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0.5688</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Achei a aula muito didática, os exemplos práticos ajudaram demais a entender o conteúdo. Valeu monitor!</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Achei a aula muito didática os exemplos práticos ajudaram demais a entender o conteúdo Valeu monitor</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>gratitude</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.9766</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Estou completamente frustrado com esse trabalho. O enunciado tá confuso e nada funciona como deveria. #desespero</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Estou completamente frustrado com esse trabalho O enunciado tá confuso e nada funciona como deveria</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>anger</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0.6840000000000001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Gente, adiando a entrega do projeto para semana que vem! Sensacional demais, deu um alívio enorme 🎉</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Gente adiando a entrega do projeto para semana que vem Sensacional demais deu um alívio enorme</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>realization</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.1977</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>O aplicativo vive travando na hora de fazer o login. Decepcionado com a última atualização.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>O aplicativo vive travando na hora de fazer o login Decepcionado com a última atualização</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>disappointment</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0.9316</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Alguém mais com dificuldade na matéria de IA? Tô achando o conteúdo bem puxado este semestre... 😔</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Alguém mais com dificuldade na matéria de IA Tô achando o conteúdo bem puxado este semestre</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0.9375</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Incrível como a comunidade se ajuda aqui! Consegui resolver o bug no código em 5 minutos. Muito obrigado a todos!</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Incrível como a comunidade se ajuda aqui Consegui resolver o bug no código em minutos Muito obrigado a todos</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>gratitude</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0.9896</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Horrível, não percam o tempo de vocês assistindo esse filme. O final não faz sentido nenhum.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Horrível não percam o tempo de vocês assistindo esse filme O final não faz sentido nenhum</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>disgust</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.8726</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tô super animado com o novo projeto da disciplina! Tem tudo pra ser uma experiência sensacional. 🚀</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Tô super animado com o novo projeto da disciplina Tem tudo pra ser uma experiência sensacional</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>excitement</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.9445</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>O filme é simplesmente espetacular! Atuações impecáveis e direção fantástica. Recomendo muito! 🎬✨</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>O filme é simplesmente espetacular Atuações impecáveis e direção fantástica Recomendo muito</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0.9883</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Péssima experiência no fórum hoje, ninguém responde minhas dúvidas e o suporte é terrível... 😡</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Péssima experiência no fórum hoje ninguém responde minhas dúvidas e o suporte é terrível</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>disgust</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.5688</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Achei a aula muito didática, os exemplos práticos ajudaram demais a entender o conteúdo. Valeu monitor!</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Achei a aula muito didática os exemplos práticos ajudaram demais a entender o conteúdo Valeu monitor</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>gratitude</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.9766</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Estou completamente frustrado com esse trabalho. O enunciado tá confuso e nada funciona como deveria. #desespero</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Estou completamente frustrado com esse trabalho O enunciado tá confuso e nada funciona como deveria</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>anger</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.6840000000000001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Gente, adiando a entrega do projeto para semana que vem! Sensacional demais, deu um alívio enorme 🎉</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Gente adiando a entrega do projeto para semana que vem Sensacional demais deu um alívio enorme</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>realization</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.1977</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>O aplicativo vive travando na hora de fazer o login. Decepcionado com a última atualização.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>O aplicativo vive travando na hora de fazer o login Decepcionado com a última atualização</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>disappointment</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0.9316</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Alguém mais com dificuldade na matéria de IA? Tô achando o conteúdo bem puxado este semestre... 😔</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Alguém mais com dificuldade na matéria de IA Tô achando o conteúdo bem puxado este semestre</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0.9375</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Incrível como a comunidade se ajuda aqui! Consegui resolver o bug no código em 5 minutos. Muito obrigado a todos!</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Incrível como a comunidade se ajuda aqui Consegui resolver o bug no código em minutos Muito obrigado a todos</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>gratitude</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.9896</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Horrível, não percam o tempo de vocês assistindo esse filme. O final não faz sentido nenhum.</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Horrível não percam o tempo de vocês assistindo esse filme O final não faz sentido nenhum</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>disgust</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0.8726</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Tô super animado com o novo projeto da disciplina! Tem tudo pra ser uma experiência sensacional. 🚀</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Tô super animado com o novo projeto da disciplina Tem tudo pra ser uma experiência sensacional</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>excitement</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0.9445</v>
       </c>
     </row>
   </sheetData>
@@ -593,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -611,21 +1163,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>disgust</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sadness</t>
+          <t>gratitude</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -635,17 +1187,57 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16.7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>curiosity</t>
+          <t>anger</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16.7</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>realization</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>disappointment</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>excitement</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: adiciona dashboard Streamlit, scraper Play Store e graficos HD com 20+ emocoes
</commit_message>
<xml_diff>
--- a/analise_forum/resultados/resultados_analise.xlsx
+++ b/analise_forum/resultados/resultados_analise.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Analise_Detalhada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Detalhado" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Resumo_Percentual" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,21 +450,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>O filme é simplesmente espetacular! Atuações impecáveis e direção fantástica. Recomendo muito! 🎬✨</t>
+          <t>nao funciona</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>O filme é simplesmente espetacular Atuações impecáveis e direção fantástica Recomendo muito</t>
+          <t>nao funciona</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>admiration</t>
+          <t>disapproval</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.9883</v>
+        <v>0.8757</v>
       </c>
     </row>
     <row r="3">
@@ -473,21 +473,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Péssima experiência no fórum hoje, ninguém responde minhas dúvidas e o suporte é terrível... 😡</t>
+          <t>Igual a todos os outros bancos, trabalha com seu dinheiro e ainda cobra por isso ! AGIOTAS MODERNOS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Péssima experiência no fórum hoje ninguém responde minhas dúvidas e o suporte é terrível</t>
+          <t>Igual a todos os outros bancos trabalha com seu dinheiro e ainda cobra por isso AGIOTAS MODERNOS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>disgust</t>
+          <t>anger</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.5688</v>
+        <v>0.761</v>
       </c>
     </row>
     <row r="4">
@@ -496,21 +496,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Achei a aula muito didática, os exemplos práticos ajudaram demais a entender o conteúdo. Valeu monitor!</t>
+          <t>perfeito</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Achei a aula muito didática os exemplos práticos ajudaram demais a entender o conteúdo Valeu monitor</t>
+          <t>perfeito</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>gratitude</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.9766</v>
+        <v>0.7755</v>
       </c>
     </row>
     <row r="5">
@@ -519,21 +519,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Estou completamente frustrado com esse trabalho. O enunciado tá confuso e nada funciona como deveria. #desespero</t>
+          <t>só falta uma aba que mostre mais específico os investimentos e os dividendos</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Estou completamente frustrado com esse trabalho O enunciado tá confuso e nada funciona como deveria</t>
+          <t>só falta uma aba que mostre mais específico os investimentos e os dividendos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>anger</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.9903</v>
       </c>
     </row>
     <row r="6">
@@ -542,21 +542,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gente, adiando a entrega do projeto para semana que vem! Sensacional demais, deu um alívio enorme 🎉</t>
+          <t>muito bom</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Gente adiando a entrega do projeto para semana que vem Sensacional demais deu um alívio enorme</t>
+          <t>muito bom</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>realization</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.1977</v>
+        <v>0.9762999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -565,21 +565,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>O aplicativo vive travando na hora de fazer o login. Decepcionado com a última atualização.</t>
+          <t>não estou conseguindo logar na minha conta, tenho que ficar reinstalando o aplicativo toda a hora...</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>O aplicativo vive travando na hora de fazer o login Decepcionado com a última atualização</t>
+          <t>não estou conseguindo logar na minha conta tenho que ficar reinstalando o aplicativo toda a hora</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>disappointment</t>
+          <t>annoyance</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.9316</v>
+        <v>0.4976</v>
       </c>
     </row>
     <row r="8">
@@ -588,21 +588,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alguém mais com dificuldade na matéria de IA? Tô achando o conteúdo bem puxado este semestre... 😔</t>
+          <t>muito boa e rápido</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Alguém mais com dificuldade na matéria de IA Tô achando o conteúdo bem puxado este semestre</t>
+          <t>muito boa e rápido</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.9375</v>
+        <v>0.9822</v>
       </c>
     </row>
     <row r="9">
@@ -611,21 +611,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Incrível como a comunidade se ajuda aqui! Consegui resolver o bug no código em 5 minutos. Muito obrigado a todos!</t>
+          <t>e muito bom</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Incrível como a comunidade se ajuda aqui Consegui resolver o bug no código em minutos Muito obrigado a todos</t>
+          <t>e muito bom</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>gratitude</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.9896</v>
+        <v>0.9775</v>
       </c>
     </row>
     <row r="10">
@@ -634,21 +634,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Horrível, não percam o tempo de vocês assistindo esse filme. O final não faz sentido nenhum.</t>
+          <t>tudo OK</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Horrível não percam o tempo de vocês assistindo esse filme O final não faz sentido nenhum</t>
+          <t>tudo OK</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>disgust</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.8726</v>
+        <v>0.9928</v>
       </c>
     </row>
     <row r="11">
@@ -657,21 +657,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tô super animado com o novo projeto da disciplina! Tem tudo pra ser uma experiência sensacional. 🚀</t>
+          <t>tentando realizar um pagamento via pix e infelizmente o sistema inoperante travando , bloqueando o envio</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tô super animado com o novo projeto da disciplina Tem tudo pra ser uma experiência sensacional</t>
+          <t>tentando realizar um pagamento via pix e infelizmente o sistema inoperante travando bloqueando o envio</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>excitement</t>
+          <t>disappointment</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.9445</v>
+        <v>0.9003</v>
       </c>
     </row>
     <row r="12">
@@ -680,12 +680,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>O filme é simplesmente espetacular! Atuações impecáveis e direção fantástica. Recomendo muito! 🎬✨</t>
+          <t>ótimo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>O filme é simplesmente espetacular Atuações impecáveis e direção fantástica Recomendo muito</t>
+          <t>ótimo</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.9883</v>
+        <v>0.9659</v>
       </c>
     </row>
     <row r="13">
@@ -703,21 +703,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Péssima experiência no fórum hoje, ninguém responde minhas dúvidas e o suporte é terrível... 😡</t>
+          <t>o APP não quer abrir. Já troquei a senha achando que tinha esquecido e nada. Só dá erro ao abrir</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Péssima experiência no fórum hoje ninguém responde minhas dúvidas e o suporte é terrível</t>
+          <t>o APP não quer abrir Já troquei a senha achando que tinha esquecido e nada Só dá erro ao abrir</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>disgust</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.5688</v>
+        <v>0.8212</v>
       </c>
     </row>
     <row r="14">
@@ -726,21 +726,21 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Achei a aula muito didática, os exemplos práticos ajudaram demais a entender o conteúdo. Valeu monitor!</t>
+          <t>descobrir um bug de chave você pode colocar chave certa copiada é colada mas o sistema pode bugar na hora de transferir e enviar para outra conta para as salvas no perfil,antes de transferir pix o nome estará tudo certo depois na hora de enviar o comprovante que estará alterado o nome do destinatário e no histórico depois 🤓</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Achei a aula muito didática os exemplos práticos ajudaram demais a entender o conteúdo Valeu monitor</t>
+          <t>descobrir um bug de chave você pode colocar chave certa copiada é colada mas o sistema pode bugar na hora de transferir e enviar para outra conta para as salvas no perfilantes de transferir pix o nome estará tudo certo depois na hora de enviar o comprovante que estará alterado o nome do destinatário e no histórico depois</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>gratitude</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.9766</v>
+        <v>0.9804</v>
       </c>
     </row>
     <row r="15">
@@ -749,21 +749,21 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Estou completamente frustrado com esse trabalho. O enunciado tá confuso e nada funciona como deveria. #desespero</t>
+          <t>muito top esse aplicativo</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Estou completamente frustrado com esse trabalho O enunciado tá confuso e nada funciona como deveria</t>
+          <t>muito top esse aplicativo</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>anger</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.9585</v>
       </c>
     </row>
     <row r="16">
@@ -772,21 +772,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gente, adiando a entrega do projeto para semana que vem! Sensacional demais, deu um alívio enorme 🎉</t>
+          <t>péssima 😔</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Gente adiando a entrega do projeto para semana que vem Sensacional demais deu um alívio enorme</t>
+          <t>péssima</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>realization</t>
+          <t>disgust</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.1977</v>
+        <v>0.2652</v>
       </c>
     </row>
     <row r="17">
@@ -795,21 +795,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>O aplicativo vive travando na hora de fazer o login. Decepcionado com a última atualização.</t>
+          <t>o Nubank é nora dez pra mim n tem melhor!❤️</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>O aplicativo vive travando na hora de fazer o login Decepcionado com a última atualização</t>
+          <t>o Nubank é nora dez pra mim n tem melhor</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>disappointment</t>
+          <t>disapproval</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.9316</v>
+        <v>0.8118</v>
       </c>
     </row>
     <row r="18">
@@ -818,21 +818,21 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alguém mais com dificuldade na matéria de IA? Tô achando o conteúdo bem puxado este semestre... 😔</t>
+          <t>recentemente esse app ta um lixo</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Alguém mais com dificuldade na matéria de IA Tô achando o conteúdo bem puxado este semestre</t>
+          <t>recentemente esse app ta um lixo</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>disgust</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.9375</v>
+        <v>0.858</v>
       </c>
     </row>
     <row r="19">
@@ -841,21 +841,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Incrível como a comunidade se ajuda aqui! Consegui resolver o bug no código em 5 minutos. Muito obrigado a todos!</t>
+          <t>ótima</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Incrível como a comunidade se ajuda aqui Consegui resolver o bug no código em minutos Muito obrigado a todos</t>
+          <t>ótima</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>gratitude</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.9896</v>
+        <v>0.9647</v>
       </c>
     </row>
     <row r="20">
@@ -864,21 +864,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Horrível, não percam o tempo de vocês assistindo esse filme. O final não faz sentido nenhum.</t>
+          <t>tem sido um dos melhores bancos na minha concepção.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Horrível não percam o tempo de vocês assistindo esse filme O final não faz sentido nenhum</t>
+          <t>tem sido um dos melhores bancos na minha concepção</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>disgust</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.8726</v>
+        <v>0.9843</v>
       </c>
     </row>
     <row r="21">
@@ -887,21 +887,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tô super animado com o novo projeto da disciplina! Tem tudo pra ser uma experiência sensacional. 🚀</t>
+          <t>aplicativo demora pra abrir</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tô super animado com o novo projeto da disciplina Tem tudo pra ser uma experiência sensacional</t>
+          <t>aplicativo demora pra abrir</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>excitement</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.9445</v>
+        <v>0.9896</v>
       </c>
     </row>
     <row r="22">
@@ -910,21 +910,21 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>O filme é simplesmente espetacular! Atuações impecáveis e direção fantástica. Recomendo muito! 🎬✨</t>
+          <t>satisfeito</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>O filme é simplesmente espetacular Atuações impecáveis e direção fantástica Recomendo muito</t>
+          <t>satisfeito</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>admiration</t>
+          <t>gratitude</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.9883</v>
+        <v>0.7447</v>
       </c>
     </row>
     <row r="23">
@@ -933,21 +933,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Péssima experiência no fórum hoje, ninguém responde minhas dúvidas e o suporte é terrível... 😡</t>
+          <t>Meu banco preferido.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Péssima experiência no fórum hoje ninguém responde minhas dúvidas e o suporte é terrível</t>
+          <t>Meu banco preferido</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>disgust</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.5688</v>
+        <v>0.5183</v>
       </c>
     </row>
     <row r="24">
@@ -956,12 +956,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Achei a aula muito didática, os exemplos práticos ajudaram demais a entender o conteúdo. Valeu monitor!</t>
+          <t>show obrigado</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Achei a aula muito didática os exemplos práticos ajudaram demais a entender o conteúdo Valeu monitor</t>
+          <t>show obrigado</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.9766</v>
+        <v>0.9823</v>
       </c>
     </row>
     <row r="25">
@@ -979,21 +979,21 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Estou completamente frustrado com esse trabalho. O enunciado tá confuso e nada funciona como deveria. #desespero</t>
+          <t>adoro essa aplicativo só estou precisando de mais limite.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Estou completamente frustrado com esse trabalho O enunciado tá confuso e nada funciona como deveria</t>
+          <t>adoro essa aplicativo só estou precisando de mais limite</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>anger</t>
+          <t>love</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.9394</v>
       </c>
     </row>
     <row r="26">
@@ -1002,21 +1002,21 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Gente, adiando a entrega do projeto para semana que vem! Sensacional demais, deu um alívio enorme 🎉</t>
+          <t>confiança e acessibilidade</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Gente adiando a entrega do projeto para semana que vem Sensacional demais deu um alívio enorme</t>
+          <t>confiança e acessibilidade</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>realization</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.1977</v>
+        <v>0.9911</v>
       </c>
     </row>
     <row r="27">
@@ -1025,21 +1025,21 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>O aplicativo vive travando na hora de fazer o login. Decepcionado com a última atualização.</t>
+          <t>bom</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>O aplicativo vive travando na hora de fazer o login Decepcionado com a última atualização</t>
+          <t>bom</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>disappointment</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.9316</v>
+        <v>0.8816000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alguém mais com dificuldade na matéria de IA? Tô achando o conteúdo bem puxado este semestre... 😔</t>
+          <t>É uma preparação p as nossas vidas, onde podemos guarda nosso dinheiro</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Alguém mais com dificuldade na matéria de IA Tô achando o conteúdo bem puxado este semestre</t>
+          <t>É uma preparação p as nossas vidas onde podemos guarda nosso dinheiro</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.9375</v>
+        <v>0.9916</v>
       </c>
     </row>
     <row r="29">
@@ -1071,21 +1071,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Incrível como a comunidade se ajuda aqui! Consegui resolver o bug no código em 5 minutos. Muito obrigado a todos!</t>
+          <t>muito bom tem vários porraos de atendimento ainda mais menores de idade podem fazer suas contas com segurança então e muito bom</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Incrível como a comunidade se ajuda aqui Consegui resolver o bug no código em minutos Muito obrigado a todos</t>
+          <t>muito bom tem vários porraos de atendimento ainda mais menores de idade podem fazer suas contas com segurança então e muito bom</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>gratitude</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.9896</v>
+        <v>0.9655</v>
       </c>
     </row>
     <row r="30">
@@ -1094,21 +1094,21 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Horrível, não percam o tempo de vocês assistindo esse filme. O final não faz sentido nenhum.</t>
+          <t>otima</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Horrível não percam o tempo de vocês assistindo esse filme O final não faz sentido nenhum</t>
+          <t>otima</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>disgust</t>
+          <t>optimism</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.8726</v>
+        <v>0.9517</v>
       </c>
     </row>
     <row r="31">
@@ -1117,21 +1117,1631 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Tô super animado com o novo projeto da disciplina! Tem tudo pra ser uma experiência sensacional. 🚀</t>
+          <t>nubank e top</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tô super animado com o novo projeto da disciplina Tem tudo pra ser uma experiência sensacional</t>
+          <t>nubank e top</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>excitement</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.9445</v>
+        <v>0.9915</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>amo muito</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>amo muito</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0.9784</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Sensacional!</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Sensacional</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0.9544</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>É bom porém não consigo acessar a conta após fazer o pagamento</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>É bom porém não consigo acessar a conta após fazer o pagamento</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0.3879</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>é um banco que confia naquele que o escolhe para abrir uma conta da oportunidade de se reerguer e aprender a usar o crédito obrigada Nubank pela confiança e credibilidade</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>é um banco que confia naquele que o escolhe para abrir uma conta da oportunidade de se reerguer e aprender a usar o crédito obrigada Nubank pela confiança e credibilidade</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>gratitude</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0.9530999999999999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Um banco que me ajuda em cada momento diferente da melhor forma.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Um banco que me ajuda em cada momento diferente da melhor forma</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>disappointment</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0.411</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Ótimo</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Ótimo</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0.9607</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>muito ótimo e excelente</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>muito ótimo e excelente</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0.9792</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>muito bom 👍</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>muito bom</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0.9762999999999999</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>péssimo app, não consegui nada nessa p</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>péssimo app não consegui nada nessa p</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>disappointment</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0.7471</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>muito bom</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>muito bom</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0.9762999999999999</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>a pessoa não consegue mandar pix para mim não sei o que tá acontecendo eu tô mandando mensagem para ele ele não atende não recomendo para ninguém</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>a pessoa não consegue mandar pix para mim não sei o que tá acontecendo eu tô mandando mensagem para ele ele não atende não recomendo para ninguém</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>disapproval</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0.8573</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>NUBANK: Quero 10mil pela minha avaliação App muito bom você só precisa de tudo e o resto</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>NUBANK Quero mil pela minha avaliação App muito bom você só precisa de tudo e o resto</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>desire</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0.708</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>gostei</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>gostei</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>joy</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0.7701</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>muito bom</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>muito bom</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0.9762999999999999</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Cobranças indevidas na fatura do cartão e péssimo suporte.</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Cobranças indevidas na fatura do cartão e péssimo suporte</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>annoyance</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0.4289</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>enrosca na abertura, na configuração e no cadastro de chave pix, "ocorreu erro"; muito esclarecedor, anos dps que eu ja baixei o, mas tudo bem espero mais alguns anos antes de aportar capital...</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>enrosca na abertura na configuração e no cadastro de chave pix ocorreu erro muito esclarecedor anos dps que eu ja baixei o mas tudo bem espero mais alguns anos antes de aportar capital</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>optimism</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0.8389</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>não deixa baixar comprovante, esses dias caiu o pix em todo o Brasil. e ainda some dinheiro da caixinha</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>não deixa baixar comprovante esses dias caiu o pix em todo o Brasil e ainda some dinheiro da caixinha</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0.8085</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>lixo vvs são uns lixos aplicativo podre não serve pra nada</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>lixo vvs são uns lixos aplicativo podre não serve pra nada</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>annoyance</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0.5849</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>mais de 4 anos com o nubank e me dá 900 reais de limite</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>mais de anos com o nubank e me dá reais de limite</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0.9774</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Eu, amei muito! 💖 💖 💖 💖 💖</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Eu amei muito</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>love</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0.9807</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Muito bom,excelente atendimento, nota 10</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Muito bomexcelente atendimento nota</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>0.9858</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>eu ❤️ ajuda muito os clientes. indiquei para vários Amigos</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>eu ajuda muito os clientes indiquei para vários Amigos</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0.5374</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>perfeito</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>perfeito</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0.7755</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Boa funcionalidade e navegação!</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Boa funcionalidade e navegação</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0.9814000000000001</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>melhor cartão de trabalhar.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>melhor cartão de trabalhar</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0.9525</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>estou me adaptando</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>estou me adaptando</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>0.993</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>estou muito satisfeito com o app</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>estou muito satisfeito com o app</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>gratitude</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>0.8871</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>excelente</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>excelente</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0.9596</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ótimo</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ótimo</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>0.9659</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>não estou conseguindo abrir o aplicativo.</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>não estou conseguindo abrir o aplicativo</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>0.7842</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>muito bom</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>muito bom</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>0.9762999999999999</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ótimo 😀</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>ótimo</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>0.9659</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Seria melhor mais sigilo.</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Seria melhor mais sigilo</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>0.9491000000000001</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>gosto muito de uza esse banco muito bom</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>gosto muito de uza esse banco muito bom</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>0.9768</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>excelente App</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>excelente App</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0.9821</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ótimo perfeito ❤️🤝</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ótimo perfeito</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>0.9758</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ótimo desempenho bom aplicativo gostei muito</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ótimo desempenho bom aplicativo gostei muito</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>0.9845</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>bom</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>bom</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>0.8816000000000001</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>muito bom mas tem um bug que sai da conta e precisa do CPF e a senha bom ele e mas no lugar que eu tava n tinha as informações e me deixou na mão tirando isso ele e incrível</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>muito bom mas tem um bug que sai da conta e precisa do CPF e a senha bom ele e mas no lugar que eu tava n tinha as informações e me deixou na mão tirando isso ele e incrível</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0.9873</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Muito Bom</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Muito Bom</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>0.9715</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>eu acho bom</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>eu acho bom</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>0.9393</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>bloquear a minha conta em menos de dois meses de uso está travado cento e pouco lá na minha conta e eu não consigo destravar a conta</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>bloquear a minha conta em menos de dois meses de uso está travado cento e pouco lá na minha conta e eu não consigo destravar a conta</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>0.7547</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>o que está acontecendo com o Pix por QR, antes tinha que ler 1 vez e lia rápido, depois 2, agora tem que ler 3 vezes pra pegar</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>o que está acontecendo com o Pix por QR antes tinha que ler vez e lia rápido depois agora tem que ler vezes pra pegar</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>0.6863</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>gostei bastante</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>gostei bastante</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>joy</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>0.8597</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>muito bom muito ativo</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>muito bom muito ativo</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>0.9715</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>péssimo horrível..... estou tentando fazer um pix N consigo N aconselho ninguém a baixar aplicativos .</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>péssimo horrível estou tentando fazer um pix N consigo N aconselho ninguém a baixar aplicativos</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>disapproval</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>0.6994</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ótimo oq n gostei e que n consigo fazer emvestimantos</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ótimo oq n gostei e que n consigo fazer emvestimantos</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>disapproval</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>0.8073</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>excelente</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>excelente</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>0.9596</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>bom</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>bom</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>0.8816000000000001</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Ótimo</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Ótimo</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>0.9607</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>muito bom não tem oq dizer tem até como mandar pix no aidio</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>muito bom não tem oq dizer tem até como mandar pix no aidio</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>0.9758</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>demoram para aumentar o limite de crédito</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>demoram para aumentar o limite de crédito</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>0.9868</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Muito boa</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Muito boa</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>0.9738</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ruim</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>ruim</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>disappointment</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>0.3962</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>muito bom</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>muito bom</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>0.9762999999999999</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>se roupa meu dinheiro eu maro</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>se roupa meu dinheiro eu maro</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>0.9788</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>muito bom ó melhor aplicativo</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>muito bom ó melhor aplicativo</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>0.9811</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Prático</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Prático</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Aplicativo bonito e fácil de utilizar. Poderiam permitir personalizar a área principal do aplicativo.</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Aplicativo bonito e fácil de utilizar Poderiam permitir personalizar a área principal do aplicativo</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>0.9787</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>eficiência</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>eficiência</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>0.9588</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>não está aparecendo a opção de entrar na minha conta.</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>não está aparecendo a opção de entrar na minha conta</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>0.9851</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>o menhor né</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>o menhor né</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>0.9846</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>porque us aplicativo não estão funcionando do. meu banco nubak. e meu ZAP e u kaui</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>porque us aplicativo não estão funcionando do meu banco nubak e meu ZAP e u kaui</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>0.3219</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>mais omenos</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>mais omenos</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>0.979</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>aplicativo ótimo, excelente atendimento</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>aplicativo ótimo excelente atendimento</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>0.9812</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>ótimo</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>ótimo</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>0.9659</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>ótima. O kit</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>ótima O kit</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>admiration</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>0.9725</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>NU Bank Sevindo o Brasil e o mundo é con muita con Pretesia e qualidade de Ademinitra cao sou DOMINGOS JORGE FARIAS CARDOSO e 👍👍👍👍👍👍👍👍👍👍👍👍👍👍👍👍</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>NU Bank Sevindo o Brasil e o mundo é con muita con Pretesia e qualidade de Ademinitra cao sou DOMINGOS JORGE FARIAS CARDOSO e</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>0.8827</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>otimo</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>otimo</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>optimism</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>0.9257</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Estou do lado do Wi-Fi. Está funcionando perfeitamente, fui tentar abrir o APP e não abre. Resolvam logo isso. Por gentileza...</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Estou do lado do WiFi Está funcionando perfeitamente fui tentar abrir o APP e não abre Resolvam logo isso Por gentileza</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>0.402</v>
       </c>
     </row>
   </sheetData>
@@ -1145,7 +2755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1156,88 +2766,169 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Porcentagem (%)</t>
+          <t>Proporcao</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Percentual</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>disgust</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>0.42</v>
+      </c>
+      <c r="C2" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>gratitude</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>0.3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>admiration</t>
+          <t>disapproval</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>0.05</v>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>anger</t>
+          <t>disappointment</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>0.04</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>realization</t>
+          <t>gratitude</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>0.04</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>disappointment</t>
+          <t>annoyance</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>0.03</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>love</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>0.03</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>excitement</t>
+          <t>optimism</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>0.03</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>disgust</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>joy</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>anger</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>desire</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>